<commit_message>
Final report submission for Group 08
</commit_message>
<xml_diff>
--- a/49K14.2_Group08_BugTrackingList.xlsx
+++ b/49K14.2_Group08_BugTrackingList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lqdvk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3398A22A-CFA2-4AE5-9596-1A03A1267289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C8AEA4-F72D-46C2-9261-72ACC2435CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Report" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="238">
   <si>
     <t>BUG TRACKING LIST</t>
   </si>
@@ -822,12 +822,15 @@
   <si>
     <t>Liên quan TC-5.1-01. Thiếu input số lượng</t>
   </si>
+  <si>
+    <t>Pass</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -908,22 +911,6 @@
     <font>
       <b/>
       <sz val="13"/>
-      <color rgb="FF38761D"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="163"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="163"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
       <color rgb="FFC00000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -933,6 +920,14 @@
       <b/>
       <sz val="13"/>
       <color rgb="FFFF6600"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF00602B"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="163"/>
@@ -1018,7 +1013,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1056,29 +1051,8 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1086,7 +1060,7 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1095,7 +1069,7 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1108,12 +1082,23 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF00602B"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1347,24 +1332,24 @@
   <sheetData>
     <row r="1" spans="1:17" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
     </row>
     <row r="2" spans="1:17" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1408,7 +1393,9 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="J3" s="8">
+        <v>19</v>
+      </c>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
@@ -1474,52 +1461,52 @@
       <c r="A5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="I5" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L5" s="17" t="s">
+      <c r="L5" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="M5" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N5" s="18">
-        <v>46144</v>
-      </c>
-      <c r="O5" s="18">
+      <c r="M5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N5" s="17">
+        <v>46135</v>
+      </c>
+      <c r="O5" s="17">
         <v>46141</v>
       </c>
-      <c r="P5" s="19" t="s">
+      <c r="P5" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q5" s="13" t="s">
+      <c r="Q5" s="24" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1527,52 +1514,52 @@
       <c r="A6" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="J6" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="M6" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N6" s="18">
-        <v>46144</v>
-      </c>
-      <c r="O6" s="18">
+      <c r="M6" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N6" s="17">
+        <v>46135</v>
+      </c>
+      <c r="O6" s="17">
         <v>46141</v>
       </c>
-      <c r="P6" s="19" t="s">
+      <c r="P6" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q6" s="13" t="s">
+      <c r="Q6" s="24" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1580,949 +1567,949 @@
       <c r="A7" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I7" s="15" t="s">
+      <c r="I7" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J7" s="20" t="s">
+      <c r="J7" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L7" s="17" t="s">
+      <c r="L7" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N7" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O7" s="18">
+      <c r="M7" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N7" s="17">
+        <v>46136</v>
+      </c>
+      <c r="O7" s="17">
         <v>46141</v>
       </c>
-      <c r="P7" s="19" t="s">
+      <c r="P7" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q7" s="13"/>
+      <c r="Q7" s="16"/>
     </row>
     <row r="8" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="20" t="s">
+      <c r="J8" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K8" s="17" t="s">
+      <c r="K8" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L8" s="17" t="s">
+      <c r="L8" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="M8" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N8" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O8" s="18">
+      <c r="M8" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N8" s="17">
+        <v>46136</v>
+      </c>
+      <c r="O8" s="17">
         <v>46141</v>
       </c>
-      <c r="P8" s="19" t="s">
+      <c r="P8" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q8" s="13"/>
+      <c r="Q8" s="16"/>
     </row>
     <row r="9" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="20" t="s">
+      <c r="J9" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K9" s="17" t="s">
+      <c r="K9" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L9" s="17" t="s">
+      <c r="L9" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="M9" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N9" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O9" s="18">
+      <c r="M9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N9" s="17">
+        <v>46136</v>
+      </c>
+      <c r="O9" s="17">
         <v>46141</v>
       </c>
-      <c r="P9" s="19" t="s">
+      <c r="P9" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q9" s="13"/>
+      <c r="Q9" s="16"/>
     </row>
     <row r="10" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J10" s="20" t="s">
+      <c r="J10" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K10" s="17" t="s">
+      <c r="K10" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L10" s="17" t="s">
+      <c r="L10" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M10" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N10" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O10" s="18">
+      <c r="M10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N10" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O10" s="17">
         <v>46141</v>
       </c>
-      <c r="P10" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q10" s="13"/>
+      <c r="P10" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q10" s="16"/>
     </row>
     <row r="11" spans="1:17" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="I11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="20" t="s">
+      <c r="J11" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K11" s="17" t="s">
+      <c r="K11" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L11" s="17" t="s">
+      <c r="L11" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M11" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N11" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O11" s="18">
+      <c r="M11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O11" s="17">
         <v>46141</v>
       </c>
-      <c r="P11" s="19" t="s">
+      <c r="P11" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q11" s="13"/>
+      <c r="Q11" s="16"/>
     </row>
     <row r="12" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="H12" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J12" s="20" t="s">
+      <c r="J12" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K12" s="17" t="s">
+      <c r="K12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L12" s="17" t="s">
+      <c r="L12" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M12" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N12" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O12" s="18">
+      <c r="M12" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N12" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O12" s="17">
         <v>46141</v>
       </c>
-      <c r="P12" s="19" t="s">
+      <c r="P12" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q12" s="13"/>
+      <c r="Q12" s="16"/>
     </row>
     <row r="13" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="H13" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J13" s="20" t="s">
+      <c r="J13" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K13" s="17" t="s">
+      <c r="K13" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L13" s="17" t="s">
+      <c r="L13" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M13" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N13" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O13" s="18">
+      <c r="M13" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N13" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O13" s="17">
         <v>46141</v>
       </c>
-      <c r="P13" s="19" t="s">
+      <c r="P13" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q13" s="13"/>
+      <c r="Q13" s="16"/>
     </row>
     <row r="14" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J14" s="20" t="s">
+      <c r="J14" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K14" s="17" t="s">
+      <c r="K14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M14" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N14" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O14" s="18">
+      <c r="M14" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N14" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O14" s="17">
         <v>46141</v>
       </c>
-      <c r="P14" s="19" t="s">
+      <c r="P14" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q14" s="13"/>
+      <c r="Q14" s="16"/>
     </row>
     <row r="15" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="G15" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J15" s="20" t="s">
+      <c r="J15" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K15" s="17" t="s">
+      <c r="K15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L15" s="17" t="s">
+      <c r="L15" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M15" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N15" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O15" s="18">
+      <c r="M15" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N15" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O15" s="17">
         <v>46141</v>
       </c>
-      <c r="P15" s="19" t="s">
+      <c r="P15" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q15" s="13"/>
+      <c r="Q15" s="16"/>
     </row>
     <row r="16" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="F16" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="H16" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J16" s="20" t="s">
+      <c r="J16" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K16" s="17" t="s">
+      <c r="K16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L16" s="17" t="s">
+      <c r="L16" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M16" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N16" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O16" s="18">
+      <c r="M16" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N16" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O16" s="17">
         <v>46141</v>
       </c>
-      <c r="P16" s="19" t="s">
+      <c r="P16" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q16" s="13"/>
+      <c r="Q16" s="16"/>
     </row>
     <row r="17" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="F17" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I17" s="15" t="s">
+      <c r="I17" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J17" s="20" t="s">
+      <c r="J17" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K17" s="17" t="s">
+      <c r="K17" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L17" s="17" t="s">
+      <c r="L17" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M17" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N17" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O17" s="18">
+      <c r="M17" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N17" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O17" s="17">
         <v>46141</v>
       </c>
-      <c r="P17" s="19" t="s">
+      <c r="P17" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q17" s="13"/>
+      <c r="Q17" s="16"/>
     </row>
     <row r="18" spans="1:17" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="15" t="s">
+      <c r="I18" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J18" s="20" t="s">
+      <c r="J18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K18" s="17" t="s">
+      <c r="K18" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L18" s="17" t="s">
+      <c r="L18" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M18" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N18" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O18" s="18">
+      <c r="M18" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N18" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O18" s="17">
         <v>46141</v>
       </c>
-      <c r="P18" s="19" t="s">
+      <c r="P18" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q18" s="13"/>
+      <c r="Q18" s="16"/>
     </row>
     <row r="19" spans="1:17" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="F19" s="13" t="s">
+      <c r="F19" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="G19" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="H19" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I19" s="15" t="s">
+      <c r="I19" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J19" s="20" t="s">
+      <c r="J19" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="K19" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L19" s="17" t="s">
+      <c r="L19" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M19" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N19" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O19" s="18">
+      <c r="M19" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N19" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O19" s="17">
         <v>46141</v>
       </c>
-      <c r="P19" s="19" t="s">
+      <c r="P19" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q19" s="13"/>
+      <c r="Q19" s="16"/>
     </row>
     <row r="20" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="F20" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="G20" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="H20" s="14" t="s">
+      <c r="H20" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="I20" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J20" s="20" t="s">
+      <c r="J20" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="K20" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L20" s="17" t="s">
+      <c r="L20" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M20" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N20" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O20" s="18">
+      <c r="M20" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N20" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O20" s="17">
         <v>46141</v>
       </c>
-      <c r="P20" s="19" t="s">
+      <c r="P20" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q20" s="13"/>
+      <c r="Q20" s="16"/>
     </row>
     <row r="21" spans="1:17" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="F21" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="H21" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J21" s="20" t="s">
+      <c r="J21" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K21" s="17" t="s">
+      <c r="K21" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L21" s="17" t="s">
+      <c r="L21" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M21" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N21" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O21" s="18">
+      <c r="M21" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N21" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O21" s="17">
         <v>46141</v>
       </c>
-      <c r="P21" s="19" t="s">
+      <c r="P21" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q21" s="13"/>
+      <c r="Q21" s="16"/>
     </row>
     <row r="22" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="H22" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="I22" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J22" s="20" t="s">
+      <c r="J22" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="K22" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L22" s="17" t="s">
+      <c r="L22" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M22" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N22" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O22" s="18">
+      <c r="M22" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N22" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O22" s="17">
         <v>46141</v>
       </c>
-      <c r="P22" s="19" t="s">
+      <c r="P22" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q22" s="13"/>
+      <c r="Q22" s="16"/>
     </row>
     <row r="23" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="F23" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="H23" s="15" t="s">
+      <c r="H23" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I23" s="15" t="s">
+      <c r="I23" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J23" s="20" t="s">
+      <c r="J23" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K23" s="17" t="s">
+      <c r="K23" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L23" s="17" t="s">
+      <c r="L23" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M23" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N23" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O23" s="18">
+      <c r="M23" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N23" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O23" s="17">
         <v>46141</v>
       </c>
-      <c r="P23" s="19" t="s">
+      <c r="P23" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q23" s="13"/>
+      <c r="Q23" s="16"/>
     </row>
     <row r="24" spans="1:17" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="F24" s="13" t="s">
+      <c r="F24" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="G24" s="13" t="s">
+      <c r="G24" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="H24" s="14" t="s">
+      <c r="H24" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="I24" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J24" s="20" t="s">
+      <c r="J24" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="K24" s="17" t="s">
+      <c r="K24" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L24" s="17" t="s">
+      <c r="L24" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M24" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="N24" s="18">
-        <v>46137</v>
-      </c>
-      <c r="O24" s="18">
+      <c r="M24" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N24" s="17">
+        <v>46138</v>
+      </c>
+      <c r="O24" s="17">
         <v>46141</v>
       </c>
-      <c r="P24" s="19" t="s">
+      <c r="P24" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="Q24" s="13"/>
+      <c r="Q24" s="16"/>
     </row>
     <row r="25" spans="1:17" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="D25" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="E25" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="G25" s="21" t="s">
+      <c r="G25" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="H25" s="22" t="s">
+      <c r="H25" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I25" s="23" t="s">
+      <c r="I25" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J25" s="16" t="s">
+      <c r="J25" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K25" s="12" t="s">
@@ -2534,48 +2521,48 @@
       <c r="M25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N25" s="24">
+      <c r="N25" s="17">
         <v>46137</v>
       </c>
-      <c r="O25" s="24" t="s">
+      <c r="O25" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P25" s="23" t="s">
+      <c r="P25" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q25" s="21" t="s">
+      <c r="Q25" s="14" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="67.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" ht="84" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="E26" s="21" t="s">
+      <c r="E26" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="F26" s="21" t="s">
+      <c r="F26" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="G26" s="21" t="s">
+      <c r="G26" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="22" t="s">
+      <c r="H26" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I26" s="22" t="s">
+      <c r="I26" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="J26" s="16" t="s">
+      <c r="J26" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K26" s="12" t="s">
@@ -2587,16 +2574,16 @@
       <c r="M26" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N26" s="24">
+      <c r="N26" s="17">
         <v>46137</v>
       </c>
-      <c r="O26" s="24" t="s">
+      <c r="O26" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P26" s="23" t="s">
+      <c r="P26" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q26" s="21" t="s">
+      <c r="Q26" s="14" t="s">
         <v>164</v>
       </c>
     </row>
@@ -2604,31 +2591,31 @@
       <c r="A27" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="E27" s="21" t="s">
+      <c r="E27" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="F27" s="21" t="s">
+      <c r="F27" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="G27" s="21" t="s">
+      <c r="G27" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="H27" s="22" t="s">
+      <c r="H27" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I27" s="23" t="s">
+      <c r="I27" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J27" s="16" t="s">
+      <c r="J27" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K27" s="12" t="s">
@@ -2640,16 +2627,16 @@
       <c r="M27" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N27" s="24">
+      <c r="N27" s="17">
         <v>46137</v>
       </c>
-      <c r="O27" s="24" t="s">
+      <c r="O27" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P27" s="23" t="s">
+      <c r="P27" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q27" s="21" t="s">
+      <c r="Q27" s="14" t="s">
         <v>171</v>
       </c>
     </row>
@@ -2657,31 +2644,31 @@
       <c r="A28" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="E28" s="21" t="s">
+      <c r="E28" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="F28" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="G28" s="21" t="s">
+      <c r="G28" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="H28" s="25" t="s">
+      <c r="H28" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I28" s="22" t="s">
+      <c r="I28" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="J28" s="16" t="s">
+      <c r="J28" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K28" s="12" t="s">
@@ -2693,16 +2680,16 @@
       <c r="M28" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N28" s="24">
+      <c r="N28" s="17">
         <v>46137</v>
       </c>
-      <c r="O28" s="24" t="s">
+      <c r="O28" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P28" s="23" t="s">
+      <c r="P28" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q28" s="21" t="s">
+      <c r="Q28" s="14" t="s">
         <v>179</v>
       </c>
     </row>
@@ -2710,31 +2697,31 @@
       <c r="A29" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="B29" s="21" t="s">
+      <c r="B29" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="E29" s="21" t="s">
+      <c r="E29" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="F29" s="21" t="s">
+      <c r="F29" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="G29" s="21" t="s">
+      <c r="G29" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="H29" s="25" t="s">
+      <c r="H29" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I29" s="25" t="s">
+      <c r="I29" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J29" s="16" t="s">
+      <c r="J29" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K29" s="12" t="s">
@@ -2746,16 +2733,16 @@
       <c r="M29" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N29" s="24">
+      <c r="N29" s="17">
         <v>46137</v>
       </c>
-      <c r="O29" s="24" t="s">
+      <c r="O29" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P29" s="23" t="s">
+      <c r="P29" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q29" s="21" t="s">
+      <c r="Q29" s="14" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2763,31 +2750,31 @@
       <c r="A30" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="E30" s="21" t="s">
+      <c r="E30" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="F30" s="21" t="s">
+      <c r="F30" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="G30" s="21" t="s">
+      <c r="G30" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="H30" s="23" t="s">
+      <c r="H30" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="I30" s="23" t="s">
+      <c r="I30" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J30" s="16" t="s">
+      <c r="J30" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K30" s="12" t="s">
@@ -2799,16 +2786,16 @@
       <c r="M30" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N30" s="24">
+      <c r="N30" s="17">
         <v>46137</v>
       </c>
-      <c r="O30" s="24" t="s">
+      <c r="O30" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P30" s="23" t="s">
+      <c r="P30" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q30" s="21" t="s">
+      <c r="Q30" s="14" t="s">
         <v>195</v>
       </c>
     </row>
@@ -2816,31 +2803,31 @@
       <c r="A31" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="C31" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="E31" s="21" t="s">
+      <c r="E31" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="F31" s="21" t="s">
+      <c r="F31" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="G31" s="21" t="s">
+      <c r="G31" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="H31" s="22" t="s">
+      <c r="H31" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I31" s="23" t="s">
+      <c r="I31" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J31" s="16" t="s">
+      <c r="J31" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K31" s="12" t="s">
@@ -2852,16 +2839,16 @@
       <c r="M31" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N31" s="24">
+      <c r="N31" s="17">
         <v>46137</v>
       </c>
-      <c r="O31" s="24" t="s">
+      <c r="O31" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P31" s="23" t="s">
+      <c r="P31" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q31" s="21" t="s">
+      <c r="Q31" s="14" t="s">
         <v>202</v>
       </c>
     </row>
@@ -2869,31 +2856,31 @@
       <c r="A32" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="D32" s="21" t="s">
+      <c r="D32" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="G32" s="21" t="s">
+      <c r="G32" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="H32" s="23" t="s">
+      <c r="H32" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="I32" s="23" t="s">
+      <c r="I32" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J32" s="16" t="s">
+      <c r="J32" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K32" s="12" t="s">
@@ -2905,16 +2892,16 @@
       <c r="M32" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N32" s="24">
+      <c r="N32" s="17">
         <v>46137</v>
       </c>
-      <c r="O32" s="24" t="s">
+      <c r="O32" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P32" s="23" t="s">
+      <c r="P32" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q32" s="21" t="s">
+      <c r="Q32" s="14" t="s">
         <v>209</v>
       </c>
     </row>
@@ -2922,31 +2909,31 @@
       <c r="A33" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="C33" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="D33" s="21" t="s">
+      <c r="D33" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="E33" s="21" t="s">
+      <c r="E33" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="F33" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="G33" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="H33" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="I33" s="23" t="s">
+      <c r="I33" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J33" s="16" t="s">
+      <c r="J33" s="13" t="s">
         <v>2</v>
       </c>
       <c r="K33" s="12" t="s">
@@ -2958,16 +2945,16 @@
       <c r="M33" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N33" s="24">
+      <c r="N33" s="17">
         <v>46137</v>
       </c>
-      <c r="O33" s="24" t="s">
+      <c r="O33" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="P33" s="23" t="s">
+      <c r="P33" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q33" s="21" t="s">
+      <c r="Q33" s="14" t="s">
         <v>217</v>
       </c>
     </row>
@@ -2975,52 +2962,52 @@
       <c r="A34" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="C34" s="21" t="s">
+      <c r="C34" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="E34" s="21" t="s">
+      <c r="E34" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="14" t="s">
         <v>223</v>
       </c>
-      <c r="G34" s="21" t="s">
+      <c r="G34" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="H34" s="22" t="s">
+      <c r="H34" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I34" s="23" t="s">
+      <c r="I34" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J34" s="16" t="s">
+      <c r="J34" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="K34" s="27" t="s">
+      <c r="K34" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="L34" s="27" t="s">
+      <c r="L34" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="M34" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="N34" s="28">
+      <c r="M34" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="N34" s="21">
         <v>45776</v>
       </c>
-      <c r="O34" s="28" t="s">
+      <c r="O34" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="P34" s="23" t="s">
+      <c r="P34" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q34" s="21" t="s">
+      <c r="Q34" s="14" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3028,52 +3015,52 @@
       <c r="A35" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="C35" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="E35" s="21" t="s">
+      <c r="E35" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="F35" s="21" t="s">
+      <c r="F35" s="14" t="s">
         <v>223</v>
       </c>
-      <c r="G35" s="21" t="s">
+      <c r="G35" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="H35" s="22" t="s">
+      <c r="H35" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I35" s="23" t="s">
+      <c r="I35" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J35" s="16" t="s">
+      <c r="J35" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="K35" s="27" t="s">
+      <c r="K35" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="L35" s="27" t="s">
+      <c r="L35" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="M35" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="N35" s="28">
+      <c r="M35" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="N35" s="21">
         <v>45776</v>
       </c>
-      <c r="O35" s="28" t="s">
+      <c r="O35" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="P35" s="23" t="s">
+      <c r="P35" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q35" s="21" t="s">
+      <c r="Q35" s="14" t="s">
         <v>230</v>
       </c>
     </row>
@@ -3081,52 +3068,52 @@
       <c r="A36" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="C36" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="E36" s="21" t="s">
+      <c r="E36" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="F36" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="G36" s="21" t="s">
+      <c r="G36" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="H36" s="22" t="s">
+      <c r="H36" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I36" s="23" t="s">
+      <c r="I36" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="J36" s="16" t="s">
+      <c r="J36" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="K36" s="27" t="s">
+      <c r="K36" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="L36" s="27" t="s">
+      <c r="L36" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="M36" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="N36" s="28">
+      <c r="M36" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="N36" s="21">
         <v>45776</v>
       </c>
-      <c r="O36" s="28" t="s">
+      <c r="O36" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="P36" s="23" t="s">
+      <c r="P36" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="Q36" s="21" t="s">
+      <c r="Q36" s="14" t="s">
         <v>236</v>
       </c>
     </row>

</xml_diff>